<commit_message>
Daily NSE scan: 2026-10-02
</commit_message>
<xml_diff>
--- a/output/2026-10-02/enriched_analysis.xlsx
+++ b/output/2026-10-02/enriched_analysis.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BR51"/>
+  <dimension ref="A1:BR50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -929,10 +929,10 @@
         </is>
       </c>
       <c r="V2" t="n">
-        <v>2.731</v>
+        <v>2.728</v>
       </c>
       <c r="W2" t="n">
-        <v>2856</v>
+        <v>2859</v>
       </c>
       <c r="X2" t="n">
         <v>22.4</v>
@@ -1396,10 +1396,10 @@
         <v>0.048</v>
       </c>
       <c r="W4" t="n">
-        <v>2769</v>
+        <v>2766</v>
       </c>
       <c r="X4" t="n">
-        <v>9.52</v>
+        <v>9.51</v>
       </c>
       <c r="Y4" t="n">
         <v>36</v>
@@ -1625,13 +1625,13 @@
         </is>
       </c>
       <c r="V5" t="n">
-        <v>1.114</v>
+        <v>1.124</v>
       </c>
       <c r="W5" t="n">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="X5" t="n">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="Y5" t="n">
         <v>22</v>
@@ -1860,10 +1860,10 @@
         <v>0.328</v>
       </c>
       <c r="W6" t="n">
-        <v>934</v>
+        <v>933</v>
       </c>
       <c r="X6" t="n">
-        <v>9.18</v>
+        <v>9.17</v>
       </c>
       <c r="Y6" t="n">
         <v>7</v>
@@ -2089,13 +2089,13 @@
         </is>
       </c>
       <c r="V7" t="n">
-        <v>1.029</v>
+        <v>1.013</v>
       </c>
       <c r="W7" t="n">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="X7" t="n">
-        <v>8.289999999999999</v>
+        <v>8.43</v>
       </c>
       <c r="Y7" t="n">
         <v>17</v>
@@ -2324,7 +2324,7 @@
         <v>0.534</v>
       </c>
       <c r="W8" t="n">
-        <v>2672</v>
+        <v>2673</v>
       </c>
       <c r="X8" t="n">
         <v>21.9</v>
@@ -2786,7 +2786,7 @@
         <v>0.063</v>
       </c>
       <c r="W10" t="n">
-        <v>1761</v>
+        <v>1759</v>
       </c>
       <c r="X10" t="n">
         <v>40.4</v>
@@ -3015,13 +3015,13 @@
         </is>
       </c>
       <c r="V11" t="n">
-        <v>0.066</v>
+        <v>0.067</v>
       </c>
       <c r="W11" t="n">
-        <v>852</v>
+        <v>846</v>
       </c>
       <c r="X11" t="n">
-        <v>21.6</v>
+        <v>21.4</v>
       </c>
       <c r="Y11" t="n">
         <v>19</v>
@@ -3248,10 +3248,10 @@
         <v>0.048</v>
       </c>
       <c r="W12" t="n">
-        <v>15098</v>
+        <v>15109</v>
       </c>
       <c r="X12" t="n">
-        <v>38.4</v>
+        <v>38.5</v>
       </c>
       <c r="Y12" t="n">
         <v>83</v>
@@ -3477,10 +3477,10 @@
         </is>
       </c>
       <c r="V13" t="n">
-        <v>0.126</v>
+        <v>0.125</v>
       </c>
       <c r="W13" t="n">
-        <v>2496</v>
+        <v>2502</v>
       </c>
       <c r="X13" t="n">
         <v>21.9</v>
@@ -3709,10 +3709,10 @@
         </is>
       </c>
       <c r="V14" t="n">
-        <v>2.296</v>
+        <v>2.286</v>
       </c>
       <c r="W14" t="n">
-        <v>2557</v>
+        <v>2568</v>
       </c>
       <c r="X14" t="n">
         <v>201</v>
@@ -3944,10 +3944,10 @@
         <v>0.124</v>
       </c>
       <c r="W15" t="n">
-        <v>693</v>
+        <v>692</v>
       </c>
       <c r="X15" t="n">
-        <v>30.2</v>
+        <v>30.1</v>
       </c>
       <c r="Y15" t="n">
         <v>17</v>
@@ -4170,7 +4170,7 @@
         <v>0.049</v>
       </c>
       <c r="W16" t="n">
-        <v>1674</v>
+        <v>1667</v>
       </c>
       <c r="X16" t="n">
         <v>22.5</v>
@@ -4399,13 +4399,13 @@
         </is>
       </c>
       <c r="V17" t="n">
-        <v>2.852</v>
+        <v>2.848</v>
       </c>
       <c r="W17" t="n">
-        <v>690</v>
+        <v>691</v>
       </c>
       <c r="X17" t="n">
-        <v>25.9</v>
+        <v>26</v>
       </c>
       <c r="Y17" t="n">
         <v>30</v>
@@ -4625,13 +4625,13 @@
         </is>
       </c>
       <c r="V18" t="n">
-        <v>0.33</v>
+        <v>0.325</v>
       </c>
       <c r="W18" t="n">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="X18" t="n">
-        <v>23.2</v>
+        <v>23.6</v>
       </c>
       <c r="Y18" t="n">
         <v>12</v>
@@ -4649,7 +4649,7 @@
         <v>7.91</v>
       </c>
       <c r="AD18" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AE18" t="b">
         <v>0</v>
@@ -4857,13 +4857,13 @@
         </is>
       </c>
       <c r="V19" t="n">
-        <v>0.37</v>
+        <v>0.371</v>
       </c>
       <c r="W19" t="n">
-        <v>1062</v>
+        <v>1060</v>
       </c>
       <c r="X19" t="n">
-        <v>54.1</v>
+        <v>54</v>
       </c>
       <c r="Y19" t="n">
         <v>21</v>
@@ -5324,7 +5324,7 @@
         <v>0.008999999999999999</v>
       </c>
       <c r="W21" t="n">
-        <v>52796</v>
+        <v>52750</v>
       </c>
       <c r="X21" t="n">
         <v>44.7</v>
@@ -5553,13 +5553,13 @@
         </is>
       </c>
       <c r="V22" t="n">
-        <v>0.2</v>
+        <v>0.191</v>
       </c>
       <c r="W22" t="n">
-        <v>555</v>
+        <v>580</v>
       </c>
       <c r="X22" t="n">
-        <v>46.3</v>
+        <v>48.5</v>
       </c>
       <c r="Y22" t="n">
         <v>3</v>
@@ -5577,7 +5577,7 @@
         <v>11.6</v>
       </c>
       <c r="AD22" t="n">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AE22" t="b">
         <v>1</v>
@@ -5788,7 +5788,7 @@
         <v>0.09</v>
       </c>
       <c r="W23" t="n">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="X23" t="n">
         <v>10.3</v>
@@ -6017,13 +6017,13 @@
         </is>
       </c>
       <c r="V24" t="n">
-        <v>0.51</v>
+        <v>0.508</v>
       </c>
       <c r="W24" t="n">
-        <v>391</v>
+        <v>393</v>
       </c>
       <c r="X24" t="n">
-        <v>36.3</v>
+        <v>36.5</v>
       </c>
       <c r="Y24" t="n">
         <v>21</v>
@@ -6249,13 +6249,13 @@
         </is>
       </c>
       <c r="V25" t="n">
-        <v>0.9399999999999999</v>
+        <v>0.931</v>
       </c>
       <c r="W25" t="n">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="X25" t="n">
-        <v>6.17</v>
+        <v>6.24</v>
       </c>
       <c r="Y25" t="n">
         <v>31</v>
@@ -6712,10 +6712,10 @@
         <v>0.233</v>
       </c>
       <c r="W27" t="n">
-        <v>600</v>
+        <v>602</v>
       </c>
       <c r="X27" t="n">
-        <v>13.2</v>
+        <v>13.3</v>
       </c>
       <c r="Y27" t="n">
         <v>-1</v>
@@ -6941,13 +6941,13 @@
         </is>
       </c>
       <c r="V28" t="n">
-        <v>0.236</v>
+        <v>0.238</v>
       </c>
       <c r="W28" t="n">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="X28" t="n">
-        <v>14.4</v>
+        <v>14.3</v>
       </c>
       <c r="Y28" t="n">
         <v>16</v>
@@ -7173,13 +7173,13 @@
         </is>
       </c>
       <c r="V29" t="n">
-        <v>0.507</v>
+        <v>0.504</v>
       </c>
       <c r="W29" t="n">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="X29" t="n">
-        <v>36.8</v>
+        <v>36.9</v>
       </c>
       <c r="Y29" t="n">
         <v>-44</v>
@@ -7408,10 +7408,10 @@
         <v>0.044</v>
       </c>
       <c r="W30" t="n">
-        <v>1572</v>
+        <v>1574</v>
       </c>
       <c r="X30" t="n">
-        <v>20.5</v>
+        <v>20.6</v>
       </c>
       <c r="Y30" t="n">
         <v>10</v>
@@ -7637,10 +7637,10 @@
         </is>
       </c>
       <c r="V31" t="n">
-        <v>0.828</v>
+        <v>0.829</v>
       </c>
       <c r="W31" t="n">
-        <v>3818</v>
+        <v>3810</v>
       </c>
       <c r="X31" t="n">
         <v>26.7</v>
@@ -7869,13 +7869,13 @@
         </is>
       </c>
       <c r="V32" t="n">
-        <v>0.658</v>
+        <v>0.65</v>
       </c>
       <c r="W32" t="n">
-        <v>357</v>
+        <v>361</v>
       </c>
       <c r="X32" t="n">
-        <v>1151</v>
+        <v>1164</v>
       </c>
       <c r="Y32" t="n">
         <v>-61</v>
@@ -8323,13 +8323,13 @@
         </is>
       </c>
       <c r="V34" t="n">
-        <v>0.363</v>
+        <v>0.366</v>
       </c>
       <c r="W34" t="n">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="X34" t="n">
-        <v>95.40000000000001</v>
+        <v>94.7</v>
       </c>
       <c r="Y34" t="n">
         <v>246</v>
@@ -8558,10 +8558,10 @@
         <v>0.23</v>
       </c>
       <c r="W35" t="n">
-        <v>1734</v>
+        <v>1733</v>
       </c>
       <c r="X35" t="n">
-        <v>18.4</v>
+        <v>18.3</v>
       </c>
       <c r="Y35" t="n">
         <v>-3</v>
@@ -8787,10 +8787,10 @@
         </is>
       </c>
       <c r="V36" t="n">
-        <v>1.96</v>
+        <v>1.909</v>
       </c>
       <c r="W36" t="n">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="X36" t="inlineStr"/>
       <c r="Y36" t="n">
@@ -9020,7 +9020,7 @@
         <v>0.042</v>
       </c>
       <c r="W37" t="n">
-        <v>3233</v>
+        <v>3230</v>
       </c>
       <c r="X37" t="n">
         <v>19.2</v>
@@ -9177,188 +9177,186 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MAHSEAMLES</t>
+          <t>INDIQUBE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Maharashtra Seamless Limited</t>
+          <t>Indiqube Spaces Limited</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>6</v>
+        <v>41</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Avoid</t>
+          <t>Watchlist</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>-1</v>
+        <v>4</v>
       </c>
       <c r="F38" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="G38" t="n">
         <v>21</v>
       </c>
       <c r="H38" t="n">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="I38" t="n">
-        <v>698.75</v>
+        <v>197.49</v>
       </c>
       <c r="J38" t="n">
-        <v>618.78</v>
+        <v>195.05</v>
       </c>
       <c r="K38" t="n">
-        <v>12.9</v>
+        <v>1.3</v>
       </c>
       <c r="L38" t="n">
-        <v>67.86</v>
+        <v>60.6</v>
       </c>
       <c r="M38" t="n">
-        <v>102.7</v>
+        <v>0.45</v>
       </c>
       <c r="N38" t="n">
-        <v>1026988804</v>
+        <v>4486152</v>
       </c>
       <c r="O38" t="n">
-        <v>1007459825</v>
+        <v>0</v>
       </c>
       <c r="P38" t="n">
-        <v>19528979</v>
+        <v>4486152</v>
       </c>
       <c r="Q38" t="n">
-        <v>98.09999999999999</v>
+        <v>0</v>
       </c>
       <c r="R38" t="inlineStr">
         <is>
-          <t>Net Buying with Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S38" t="b">
         <v>0</v>
       </c>
       <c r="T38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-09-2026</t>
         </is>
       </c>
       <c r="V38" t="n">
-        <v>0.021</v>
+        <v>0.011</v>
       </c>
       <c r="W38" t="n">
-        <v>9358</v>
-      </c>
-      <c r="X38" t="n">
-        <v>12.4</v>
-      </c>
+        <v>4187</v>
+      </c>
+      <c r="X38" t="inlineStr"/>
       <c r="Y38" t="n">
-        <v>-12</v>
+        <v>39</v>
       </c>
       <c r="Z38" t="n">
-        <v>184</v>
+        <v>258</v>
       </c>
       <c r="AA38" t="n">
-        <v>-15</v>
+        <v>30</v>
       </c>
       <c r="AB38" t="n">
-        <v>20.21</v>
+        <v>-1.13</v>
       </c>
       <c r="AC38" t="n">
-        <v>13.8</v>
+        <v>6.38</v>
       </c>
       <c r="AD38" t="n">
-        <v>0</v>
+        <v>10.11</v>
       </c>
       <c r="AE38" t="b">
         <v>1</v>
       </c>
       <c r="AF38" t="n">
-        <v>17</v>
+        <v>61</v>
       </c>
       <c r="AG38" t="n">
-        <v>646.3099999999999</v>
+        <v>189.32</v>
       </c>
       <c r="AH38" t="n">
-        <v>598.92</v>
+        <v>176.66</v>
       </c>
       <c r="AI38" t="n">
-        <v>24.7</v>
+        <v>45.6</v>
       </c>
       <c r="AJ38" t="n">
-        <v>618.7797818882931</v>
+        <v>195.0500869565217</v>
       </c>
       <c r="AK38" t="n">
-        <v>12.9</v>
+        <v>1.3</v>
       </c>
       <c r="AL38" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM38" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AN38" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Early Accumulation</t>
         </is>
       </c>
       <c r="AO38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>22-09-2026</t>
         </is>
       </c>
       <c r="AP38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-09-2026</t>
         </is>
       </c>
       <c r="AQ38" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AR38" t="n">
-        <v>94</v>
+        <v>10</v>
       </c>
       <c r="AS38" t="n">
-        <v>94</v>
+        <v>7</v>
       </c>
       <c r="AT38" t="n">
         <v>0</v>
       </c>
       <c r="AU38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AV38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AW38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AX38" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AY38" t="n">
         <v>0</v>
       </c>
       <c r="AZ38" t="n">
-        <v>0</v>
+        <v>4486152</v>
       </c>
       <c r="BA38" t="n">
-        <v>0</v>
+        <v>4486152</v>
       </c>
       <c r="BB38" t="n">
-        <v>0</v>
+        <v>4486152</v>
       </c>
       <c r="BC38" t="n">
-        <v>0</v>
+        <v>4486152</v>
       </c>
       <c r="BD38" t="n">
         <v>0</v>
@@ -9394,13 +9392,13 @@
         <v>0</v>
       </c>
       <c r="BO38" t="n">
-        <v>0</v>
+        <v>4486152</v>
       </c>
       <c r="BP38" t="n">
         <v>1</v>
       </c>
       <c r="BQ38" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR38" t="n">
         <v>0</v>
@@ -9409,57 +9407,57 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>INDIQUBE</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Indiqube Spaces Limited</t>
+          <t>U. Y. Fincorp Limited</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>41</v>
+        <v>34</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Watchlist</t>
+          <t>Fundamental Watch</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="F39" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="G39" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H39" t="n">
         <v>0</v>
       </c>
       <c r="I39" t="n">
-        <v>197.49</v>
+        <v>22.86</v>
       </c>
       <c r="J39" t="n">
-        <v>195.05</v>
+        <v>21.01</v>
       </c>
       <c r="K39" t="n">
-        <v>1.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="L39" t="n">
-        <v>60.6</v>
+        <v>70.87</v>
       </c>
       <c r="M39" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="N39" t="n">
-        <v>4486152</v>
+        <v>4960333</v>
       </c>
       <c r="O39" t="n">
         <v>0</v>
       </c>
       <c r="P39" t="n">
-        <v>4486152</v>
+        <v>4960333</v>
       </c>
       <c r="Q39" t="n">
         <v>0</v>
@@ -9473,122 +9471,120 @@
         <v>0</v>
       </c>
       <c r="T39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U39" t="inlineStr">
         <is>
-          <t>25-09-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="V39" t="n">
-        <v>0.011</v>
+        <v>0.114</v>
       </c>
       <c r="W39" t="n">
-        <v>4162</v>
-      </c>
-      <c r="X39" t="inlineStr"/>
+        <v>435</v>
+      </c>
+      <c r="X39" t="n">
+        <v>7.02</v>
+      </c>
       <c r="Y39" t="n">
-        <v>39</v>
-      </c>
-      <c r="Z39" t="n">
-        <v>258</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="Z39" t="inlineStr"/>
       <c r="AA39" t="n">
-        <v>30</v>
+        <v>391</v>
       </c>
       <c r="AB39" t="n">
-        <v>-1.13</v>
+        <v>1.03</v>
       </c>
       <c r="AC39" t="n">
-        <v>6.38</v>
+        <v>19.9</v>
       </c>
       <c r="AD39" t="n">
-        <v>10.11</v>
+        <v>0.01</v>
       </c>
       <c r="AE39" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF39" t="n">
-        <v>61</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="AF39" t="inlineStr"/>
       <c r="AG39" t="n">
-        <v>189.32</v>
+        <v>19.85</v>
       </c>
       <c r="AH39" t="n">
-        <v>176.66</v>
+        <v>15.62</v>
       </c>
       <c r="AI39" t="n">
-        <v>45.6</v>
+        <v>97.40000000000001</v>
       </c>
       <c r="AJ39" t="n">
-        <v>195.0500869565217</v>
+        <v>21.00741139152052</v>
       </c>
       <c r="AK39" t="n">
-        <v>1.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="AL39" t="inlineStr">
         <is>
-          <t>Fresh</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM39" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN39" t="inlineStr">
         <is>
-          <t>Early Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO39" t="inlineStr">
         <is>
-          <t>22-09-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="AP39" t="inlineStr">
         <is>
-          <t>25-09-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
       <c r="AQ39" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR39" t="n">
+        <v>46</v>
+      </c>
+      <c r="AS39" t="n">
+        <v>44</v>
+      </c>
+      <c r="AT39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV39" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW39" t="n">
         <v>3</v>
       </c>
-      <c r="AR39" t="n">
-        <v>10</v>
-      </c>
-      <c r="AS39" t="n">
-        <v>7</v>
-      </c>
-      <c r="AT39" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU39" t="n">
-        <v>4</v>
-      </c>
-      <c r="AV39" t="n">
-        <v>4</v>
-      </c>
-      <c r="AW39" t="n">
-        <v>4</v>
-      </c>
       <c r="AX39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AY39" t="n">
         <v>0</v>
       </c>
       <c r="AZ39" t="n">
-        <v>4486152</v>
+        <v>0</v>
       </c>
       <c r="BA39" t="n">
-        <v>4486152</v>
+        <v>0</v>
       </c>
       <c r="BB39" t="n">
-        <v>4486152</v>
+        <v>4960333</v>
       </c>
       <c r="BC39" t="n">
-        <v>4486152</v>
+        <v>4960333</v>
       </c>
       <c r="BD39" t="n">
         <v>0</v>
@@ -9624,7 +9620,7 @@
         <v>0</v>
       </c>
       <c r="BO39" t="n">
-        <v>4486152</v>
+        <v>0</v>
       </c>
       <c r="BP39" t="n">
         <v>1</v>
@@ -9639,16 +9635,16 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>U. Y. Fincorp Limited</t>
+          <t>Savita Oil Technologies Limited</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -9656,209 +9652,213 @@
         </is>
       </c>
       <c r="E40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F40" t="n">
+        <v>26</v>
+      </c>
+      <c r="G40" t="n">
+        <v>21</v>
+      </c>
+      <c r="H40" t="n">
+        <v>-13</v>
+      </c>
+      <c r="I40" t="n">
+        <v>729.5</v>
+      </c>
+      <c r="J40" t="n">
+        <v>726.25</v>
+      </c>
+      <c r="K40" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="L40" t="n">
+        <v>71.92</v>
+      </c>
+      <c r="M40" t="n">
+        <v>3.76</v>
+      </c>
+      <c r="N40" t="n">
+        <v>37641643</v>
+      </c>
+      <c r="O40" t="n">
+        <v>37427640</v>
+      </c>
+      <c r="P40" t="n">
+        <v>214003</v>
+      </c>
+      <c r="Q40" t="n">
+        <v>99.43000000000001</v>
+      </c>
+      <c r="R40" t="inlineStr">
+        <is>
+          <t>Net Buying with Selling</t>
+        </is>
+      </c>
+      <c r="S40" t="b">
+        <v>0</v>
+      </c>
+      <c r="T40" t="n">
+        <v>2</v>
+      </c>
+      <c r="U40" t="inlineStr">
+        <is>
+          <t>24-09-2026</t>
+        </is>
+      </c>
+      <c r="V40" t="n">
+        <v>0</v>
+      </c>
+      <c r="W40" t="n">
+        <v>5001</v>
+      </c>
+      <c r="X40" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="Y40" t="n">
+        <v>26</v>
+      </c>
+      <c r="Z40" t="n">
+        <v>364</v>
+      </c>
+      <c r="AA40" t="n">
+        <v>204</v>
+      </c>
+      <c r="AB40" t="n">
+        <v>42.63</v>
+      </c>
+      <c r="AC40" t="n">
         <v>14</v>
       </c>
-      <c r="G40" t="n">
+      <c r="AD40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AE40" t="b">
+        <v>1</v>
+      </c>
+      <c r="AF40" t="n">
         <v>25</v>
       </c>
-      <c r="H40" t="n">
-        <v>0</v>
-      </c>
-      <c r="I40" t="n">
-        <v>22.86</v>
-      </c>
-      <c r="J40" t="n">
-        <v>21.01</v>
-      </c>
-      <c r="K40" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="L40" t="n">
-        <v>70.87</v>
-      </c>
-      <c r="M40" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N40" t="n">
-        <v>4960333</v>
-      </c>
-      <c r="O40" t="n">
-        <v>0</v>
-      </c>
-      <c r="P40" t="n">
-        <v>4960333</v>
-      </c>
-      <c r="Q40" t="n">
-        <v>0</v>
-      </c>
-      <c r="R40" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S40" t="b">
-        <v>0</v>
-      </c>
-      <c r="T40" t="n">
-        <v>3</v>
-      </c>
-      <c r="U40" t="inlineStr">
-        <is>
-          <t>19-08-2026</t>
-        </is>
-      </c>
-      <c r="V40" t="n">
-        <v>0.115</v>
-      </c>
-      <c r="W40" t="n">
-        <v>433</v>
-      </c>
-      <c r="X40" t="n">
-        <v>6.99</v>
-      </c>
-      <c r="Y40" t="n">
-        <v>118</v>
-      </c>
-      <c r="Z40" t="inlineStr"/>
-      <c r="AA40" t="n">
-        <v>391</v>
-      </c>
-      <c r="AB40" t="n">
-        <v>1.03</v>
-      </c>
-      <c r="AC40" t="n">
-        <v>19.9</v>
-      </c>
-      <c r="AD40" t="n">
-        <v>0.01</v>
-      </c>
-      <c r="AE40" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF40" t="inlineStr"/>
       <c r="AG40" t="n">
-        <v>19.85</v>
+        <v>692.97</v>
       </c>
       <c r="AH40" t="n">
-        <v>15.62</v>
+        <v>484.19</v>
       </c>
       <c r="AI40" t="n">
-        <v>97.40000000000001</v>
+        <v>153.2</v>
       </c>
       <c r="AJ40" t="n">
-        <v>21.00741139152052</v>
+        <v>726.2520355006753</v>
       </c>
       <c r="AK40" t="n">
-        <v>8.800000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="AL40" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM40" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN40" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO40" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AP40" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
       <c r="AQ40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR40" t="n">
+        <v>8</v>
+      </c>
+      <c r="AS40" t="n">
+        <v>8</v>
+      </c>
+      <c r="AT40" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU40" t="n">
         <v>2</v>
       </c>
-      <c r="AR40" t="n">
-        <v>46</v>
-      </c>
-      <c r="AS40" t="n">
-        <v>44</v>
-      </c>
-      <c r="AT40" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU40" t="n">
-        <v>0</v>
-      </c>
       <c r="AV40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AX40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AY40" t="n">
         <v>0</v>
       </c>
       <c r="AZ40" t="n">
-        <v>0</v>
+        <v>37641643</v>
       </c>
       <c r="BA40" t="n">
-        <v>0</v>
+        <v>37641643</v>
       </c>
       <c r="BB40" t="n">
-        <v>4960333</v>
+        <v>37641643</v>
       </c>
       <c r="BC40" t="n">
-        <v>4960333</v>
+        <v>37641643</v>
       </c>
       <c r="BD40" t="n">
         <v>0</v>
       </c>
       <c r="BE40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BF40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BH40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BI40" t="n">
         <v>0</v>
       </c>
       <c r="BJ40" t="n">
-        <v>0</v>
+        <v>37427640</v>
       </c>
       <c r="BK40" t="n">
-        <v>0</v>
+        <v>37427640</v>
       </c>
       <c r="BL40" t="n">
-        <v>0</v>
+        <v>37427640</v>
       </c>
       <c r="BM40" t="n">
-        <v>0</v>
+        <v>37427640</v>
       </c>
       <c r="BN40" t="n">
         <v>0</v>
       </c>
       <c r="BO40" t="n">
-        <v>0</v>
+        <v>214003</v>
       </c>
       <c r="BP40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="BQ40" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BR40" t="n">
         <v>0</v>
@@ -9867,230 +9867,230 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Savita Oil Technologies Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Fundamental Watch</t>
+          <t>Avoid</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F41" t="n">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="G41" t="n">
         <v>21</v>
       </c>
       <c r="H41" t="n">
-        <v>-13</v>
+        <v>0</v>
       </c>
       <c r="I41" t="n">
-        <v>729.5</v>
+        <v>371.25</v>
       </c>
       <c r="J41" t="n">
-        <v>726.25</v>
+        <v>338.1</v>
       </c>
       <c r="K41" t="n">
-        <v>0.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="L41" t="n">
-        <v>71.92</v>
+        <v>66.73</v>
       </c>
       <c r="M41" t="n">
-        <v>3.76</v>
+        <v>0.34</v>
       </c>
       <c r="N41" t="n">
-        <v>37641643</v>
+        <v>3381000</v>
       </c>
       <c r="O41" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="P41" t="n">
-        <v>214003</v>
+        <v>3381000</v>
       </c>
       <c r="Q41" t="n">
-        <v>99.43000000000001</v>
+        <v>0</v>
       </c>
       <c r="R41" t="inlineStr">
         <is>
-          <t>Net Buying with Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S41" t="b">
         <v>0</v>
       </c>
       <c r="T41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U41" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="V41" t="n">
-        <v>0</v>
+        <v>0.077</v>
       </c>
       <c r="W41" t="n">
-        <v>4998</v>
+        <v>438</v>
       </c>
       <c r="X41" t="n">
-        <v>11.7</v>
+        <v>12.9</v>
       </c>
       <c r="Y41" t="n">
-        <v>26</v>
+        <v>-8</v>
       </c>
       <c r="Z41" t="n">
-        <v>364</v>
+        <v>24</v>
       </c>
       <c r="AA41" t="n">
-        <v>204</v>
+        <v>33</v>
       </c>
       <c r="AB41" t="n">
-        <v>42.63</v>
+        <v>14.36</v>
       </c>
       <c r="AC41" t="n">
-        <v>14</v>
+        <v>9.94</v>
       </c>
       <c r="AD41" t="n">
-        <v>0</v>
+        <v>0.23</v>
       </c>
       <c r="AE41" t="b">
         <v>1</v>
       </c>
       <c r="AF41" t="n">
-        <v>25</v>
+        <v>18</v>
       </c>
       <c r="AG41" t="n">
-        <v>692.97</v>
+        <v>368.17</v>
       </c>
       <c r="AH41" t="n">
-        <v>484.19</v>
+        <v>272.69</v>
       </c>
       <c r="AI41" t="n">
-        <v>153.2</v>
+        <v>99.09999999999999</v>
       </c>
       <c r="AJ41" t="n">
-        <v>726.2520355006753</v>
+        <v>338.1</v>
       </c>
       <c r="AK41" t="n">
-        <v>0.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="AL41" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Aging</t>
         </is>
       </c>
       <c r="AM41" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature Accumulation</t>
         </is>
       </c>
       <c r="AN41" t="inlineStr">
         <is>
-          <t>Confirmed Accumulation</t>
+          <t>Mature — Wait for Pullback</t>
         </is>
       </c>
       <c r="AO41" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AP41" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
       <c r="AQ41" t="n">
         <v>0</v>
       </c>
       <c r="AR41" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="AS41" t="n">
-        <v>8</v>
+        <v>52</v>
       </c>
       <c r="AT41" t="n">
         <v>0</v>
       </c>
       <c r="AU41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AV41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AW41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AX41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AY41" t="n">
         <v>0</v>
       </c>
       <c r="AZ41" t="n">
-        <v>37641643</v>
+        <v>0</v>
       </c>
       <c r="BA41" t="n">
-        <v>37641643</v>
+        <v>0</v>
       </c>
       <c r="BB41" t="n">
-        <v>37641643</v>
+        <v>3381000</v>
       </c>
       <c r="BC41" t="n">
-        <v>37641643</v>
+        <v>3381000</v>
       </c>
       <c r="BD41" t="n">
         <v>0</v>
       </c>
       <c r="BE41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BF41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BG41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BH41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BI41" t="n">
         <v>0</v>
       </c>
       <c r="BJ41" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BK41" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BL41" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BM41" t="n">
-        <v>37427640</v>
+        <v>0</v>
       </c>
       <c r="BN41" t="n">
         <v>0</v>
       </c>
       <c r="BO41" t="n">
-        <v>214003</v>
+        <v>0</v>
       </c>
       <c r="BP41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ41" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BR41" t="n">
         <v>0</v>
@@ -10099,16 +10099,16 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
@@ -10116,40 +10116,40 @@
         </is>
       </c>
       <c r="E42" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="F42" t="n">
-        <v>15</v>
+        <v>4</v>
       </c>
       <c r="G42" t="n">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="H42" t="n">
         <v>0</v>
       </c>
       <c r="I42" t="n">
-        <v>371.25</v>
+        <v>33.3</v>
       </c>
       <c r="J42" t="n">
-        <v>338.1</v>
+        <v>23.55</v>
       </c>
       <c r="K42" t="n">
-        <v>9.800000000000001</v>
+        <v>41.4</v>
       </c>
       <c r="L42" t="n">
-        <v>66.73</v>
+        <v>68.34</v>
       </c>
       <c r="M42" t="n">
-        <v>0.34</v>
+        <v>0.2</v>
       </c>
       <c r="N42" t="n">
-        <v>3381000</v>
+        <v>2018403</v>
       </c>
       <c r="O42" t="n">
         <v>0</v>
       </c>
       <c r="P42" t="n">
-        <v>3381000</v>
+        <v>2018403</v>
       </c>
       <c r="Q42" t="n">
         <v>0</v>
@@ -10163,124 +10163,124 @@
         <v>0</v>
       </c>
       <c r="T42" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="U42" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="V42" t="n">
-        <v>0.078</v>
+        <v>0.119</v>
       </c>
       <c r="W42" t="n">
-        <v>436</v>
+        <v>170</v>
       </c>
       <c r="X42" t="n">
-        <v>12.9</v>
+        <v>39.4</v>
       </c>
       <c r="Y42" t="n">
-        <v>-8</v>
+        <v>19</v>
       </c>
       <c r="Z42" t="n">
-        <v>24</v>
+        <v>3.17</v>
       </c>
       <c r="AA42" t="n">
-        <v>33</v>
+        <v>7</v>
       </c>
       <c r="AB42" t="n">
-        <v>14.36</v>
+        <v>0.49</v>
       </c>
       <c r="AC42" t="n">
-        <v>9.94</v>
+        <v>8.76</v>
       </c>
       <c r="AD42" t="n">
-        <v>0.23</v>
+        <v>0.2</v>
       </c>
       <c r="AE42" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF42" t="n">
-        <v>18</v>
+        <v>14.87</v>
       </c>
       <c r="AG42" t="n">
-        <v>368.17</v>
+        <v>23.99</v>
       </c>
       <c r="AH42" t="n">
-        <v>272.69</v>
+        <v>22.82</v>
       </c>
       <c r="AI42" t="n">
-        <v>99.09999999999999</v>
+        <v>98.8</v>
       </c>
       <c r="AJ42" t="n">
-        <v>338.1</v>
+        <v>23.5472893358377</v>
       </c>
       <c r="AK42" t="n">
-        <v>9.800000000000001</v>
+        <v>41.4</v>
       </c>
       <c r="AL42" t="inlineStr">
         <is>
-          <t>Aging</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM42" t="inlineStr">
         <is>
-          <t>Mature Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN42" t="inlineStr">
         <is>
-          <t>Mature — Wait for Pullback</t>
+          <t>Late — Poor Entry</t>
         </is>
       </c>
       <c r="AO42" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>20-08-2026</t>
         </is>
       </c>
       <c r="AP42" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
       <c r="AQ42" t="n">
-        <v>0</v>
+        <v>34</v>
       </c>
       <c r="AR42" t="n">
-        <v>52</v>
+        <v>43</v>
       </c>
       <c r="AS42" t="n">
-        <v>52</v>
+        <v>9</v>
       </c>
       <c r="AT42" t="n">
         <v>0</v>
       </c>
       <c r="AU42" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AV42" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AW42" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="AX42" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="AY42" t="n">
         <v>0</v>
       </c>
       <c r="AZ42" t="n">
-        <v>0</v>
+        <v>427686</v>
       </c>
       <c r="BA42" t="n">
-        <v>0</v>
+        <v>1399665</v>
       </c>
       <c r="BB42" t="n">
-        <v>3381000</v>
+        <v>2018403</v>
       </c>
       <c r="BC42" t="n">
-        <v>3381000</v>
+        <v>2018403</v>
       </c>
       <c r="BD42" t="n">
         <v>0</v>
@@ -10316,10 +10316,10 @@
         <v>0</v>
       </c>
       <c r="BO42" t="n">
-        <v>0</v>
+        <v>1399665</v>
       </c>
       <c r="BP42" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="BQ42" t="n">
         <v>0</v>
@@ -10331,16 +10331,16 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
@@ -10348,40 +10348,40 @@
         </is>
       </c>
       <c r="E43" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="F43" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G43" t="n">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="H43" t="n">
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="I43" t="n">
-        <v>33.3</v>
+        <v>177.64</v>
       </c>
       <c r="J43" t="n">
-        <v>23.55</v>
+        <v>170.45</v>
       </c>
       <c r="K43" t="n">
-        <v>41.4</v>
+        <v>4.2</v>
       </c>
       <c r="L43" t="n">
-        <v>68.34</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="M43" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="N43" t="n">
-        <v>2018403</v>
+        <v>2560187</v>
       </c>
       <c r="O43" t="n">
         <v>0</v>
       </c>
       <c r="P43" t="n">
-        <v>2018403</v>
+        <v>2560187</v>
       </c>
       <c r="Q43" t="n">
         <v>0</v>
@@ -10395,60 +10395,60 @@
         <v>0</v>
       </c>
       <c r="T43" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="U43" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V43" t="n">
-        <v>0.119</v>
+        <v>0.107</v>
       </c>
       <c r="W43" t="n">
-        <v>170</v>
+        <v>239</v>
       </c>
       <c r="X43" t="n">
-        <v>39.4</v>
+        <v>25.6</v>
       </c>
       <c r="Y43" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="Z43" t="n">
-        <v>3.17</v>
+        <v>1.87</v>
       </c>
       <c r="AA43" t="n">
-        <v>7</v>
+        <v>-31</v>
       </c>
       <c r="AB43" t="n">
-        <v>0.49</v>
+        <v>3.36</v>
       </c>
       <c r="AC43" t="n">
-        <v>8.76</v>
+        <v>4.96</v>
       </c>
       <c r="AD43" t="n">
-        <v>0.2</v>
+        <v>-0</v>
       </c>
       <c r="AE43" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF43" t="n">
-        <v>14.87</v>
+        <v>2.97</v>
       </c>
       <c r="AG43" t="n">
-        <v>23.99</v>
+        <v>181.33</v>
       </c>
       <c r="AH43" t="n">
-        <v>22.82</v>
+        <v>164.23</v>
       </c>
       <c r="AI43" t="n">
-        <v>98.8</v>
+        <v>66.5</v>
       </c>
       <c r="AJ43" t="n">
-        <v>23.5472893358377</v>
+        <v>170.4518641810919</v>
       </c>
       <c r="AK43" t="n">
-        <v>41.4</v>
+        <v>4.2</v>
       </c>
       <c r="AL43" t="inlineStr">
         <is>
@@ -10462,57 +10462,57 @@
       </c>
       <c r="AN43" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO43" t="inlineStr">
         <is>
-          <t>20-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP43" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ43" t="n">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="AR43" t="n">
-        <v>43</v>
+        <v>29</v>
       </c>
       <c r="AS43" t="n">
-        <v>9</v>
+        <v>29</v>
       </c>
       <c r="AT43" t="n">
         <v>0</v>
       </c>
       <c r="AU43" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="AV43" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="AW43" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="AX43" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="AY43" t="n">
         <v>0</v>
       </c>
       <c r="AZ43" t="n">
-        <v>427686</v>
+        <v>0</v>
       </c>
       <c r="BA43" t="n">
-        <v>1399665</v>
+        <v>2560187</v>
       </c>
       <c r="BB43" t="n">
-        <v>2018403</v>
+        <v>2560187</v>
       </c>
       <c r="BC43" t="n">
-        <v>2018403</v>
+        <v>2560187</v>
       </c>
       <c r="BD43" t="n">
         <v>0</v>
@@ -10548,10 +10548,10 @@
         <v>0</v>
       </c>
       <c r="BO43" t="n">
-        <v>1399665</v>
+        <v>2560187</v>
       </c>
       <c r="BP43" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="BQ43" t="n">
         <v>0</v>
@@ -10563,16 +10563,16 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -10580,40 +10580,40 @@
         </is>
       </c>
       <c r="E44" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="F44" t="n">
-        <v>8</v>
+        <v>-5</v>
       </c>
       <c r="G44" t="n">
         <v>17</v>
       </c>
       <c r="H44" t="n">
-        <v>-1</v>
+        <v>0</v>
       </c>
       <c r="I44" t="n">
-        <v>177.64</v>
+        <v>613.85</v>
       </c>
       <c r="J44" t="n">
-        <v>170.45</v>
+        <v>622.4400000000001</v>
       </c>
       <c r="K44" t="n">
-        <v>4.2</v>
+        <v>-1.4</v>
       </c>
       <c r="L44" t="n">
-        <v>67.54000000000001</v>
+        <v>74.02</v>
       </c>
       <c r="M44" t="n">
-        <v>0.26</v>
+        <v>0.49</v>
       </c>
       <c r="N44" t="n">
-        <v>2560187</v>
+        <v>4930931</v>
       </c>
       <c r="O44" t="n">
         <v>0</v>
       </c>
       <c r="P44" t="n">
-        <v>2560187</v>
+        <v>4930931</v>
       </c>
       <c r="Q44" t="n">
         <v>0</v>
@@ -10627,64 +10627,62 @@
         <v>0</v>
       </c>
       <c r="T44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="U44" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="V44" t="n">
-        <v>0.108</v>
+        <v>0.052</v>
       </c>
       <c r="W44" t="n">
-        <v>237</v>
-      </c>
-      <c r="X44" t="n">
-        <v>25.4</v>
-      </c>
+        <v>954</v>
+      </c>
+      <c r="X44" t="inlineStr"/>
       <c r="Y44" t="n">
-        <v>24</v>
+        <v>-2</v>
       </c>
       <c r="Z44" t="n">
-        <v>1.87</v>
+        <v>5</v>
       </c>
       <c r="AA44" t="n">
-        <v>-31</v>
+        <v>-152</v>
       </c>
       <c r="AB44" t="n">
-        <v>3.36</v>
+        <v>-6.5</v>
       </c>
       <c r="AC44" t="n">
-        <v>4.96</v>
+        <v>9.24</v>
       </c>
       <c r="AD44" t="n">
-        <v>-0</v>
+        <v>2.23</v>
       </c>
       <c r="AE44" t="b">
         <v>1</v>
       </c>
       <c r="AF44" t="n">
-        <v>2.97</v>
+        <v>6</v>
       </c>
       <c r="AG44" t="n">
-        <v>181.33</v>
+        <v>599.03</v>
       </c>
       <c r="AH44" t="n">
-        <v>164.23</v>
+        <v>549.9</v>
       </c>
       <c r="AI44" t="n">
-        <v>66.5</v>
+        <v>28.5</v>
       </c>
       <c r="AJ44" t="n">
-        <v>170.4518641810919</v>
+        <v>622.4351173945973</v>
       </c>
       <c r="AK44" t="n">
-        <v>4.2</v>
+        <v>-1.4</v>
       </c>
       <c r="AL44" t="inlineStr">
         <is>
-          <t>Active</t>
+          <t>Fresh</t>
         </is>
       </c>
       <c r="AM44" t="inlineStr">
@@ -10699,52 +10697,52 @@
       </c>
       <c r="AO44" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>28-08-2026</t>
         </is>
       </c>
       <c r="AP44" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
       <c r="AQ44" t="n">
-        <v>0</v>
+        <v>33</v>
       </c>
       <c r="AR44" t="n">
-        <v>29</v>
+        <v>35</v>
       </c>
       <c r="AS44" t="n">
-        <v>29</v>
+        <v>2</v>
       </c>
       <c r="AT44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AV44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AW44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AX44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="AY44" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="AZ44" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="BA44" t="n">
-        <v>2560187</v>
+        <v>3760931</v>
       </c>
       <c r="BB44" t="n">
-        <v>2560187</v>
+        <v>4930931</v>
       </c>
       <c r="BC44" t="n">
-        <v>2560187</v>
+        <v>4930931</v>
       </c>
       <c r="BD44" t="n">
         <v>0</v>
@@ -10777,34 +10775,34 @@
         <v>0</v>
       </c>
       <c r="BN44" t="n">
-        <v>0</v>
+        <v>2472736</v>
       </c>
       <c r="BO44" t="n">
-        <v>2560187</v>
+        <v>3760931</v>
       </c>
       <c r="BP44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BQ44" t="n">
         <v>0</v>
       </c>
       <c r="BR44" t="n">
-        <v>0</v>
+        <v>0.6575</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
@@ -10812,40 +10810,40 @@
         </is>
       </c>
       <c r="E45" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F45" t="n">
-        <v>-5</v>
+        <v>15</v>
       </c>
       <c r="G45" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H45" t="n">
         <v>0</v>
       </c>
       <c r="I45" t="n">
-        <v>613.85</v>
+        <v>317.4</v>
       </c>
       <c r="J45" t="n">
-        <v>622.4400000000001</v>
+        <v>335.41</v>
       </c>
       <c r="K45" t="n">
-        <v>-1.4</v>
+        <v>-5.4</v>
       </c>
       <c r="L45" t="n">
-        <v>74.02</v>
+        <v>68.48</v>
       </c>
       <c r="M45" t="n">
-        <v>0.49</v>
+        <v>0.41</v>
       </c>
       <c r="N45" t="n">
-        <v>4930931</v>
+        <v>4081958</v>
       </c>
       <c r="O45" t="n">
         <v>0</v>
       </c>
       <c r="P45" t="n">
-        <v>4930931</v>
+        <v>4081958</v>
       </c>
       <c r="Q45" t="n">
         <v>0</v>
@@ -10859,182 +10857,184 @@
         <v>0</v>
       </c>
       <c r="T45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="U45" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
       <c r="V45" t="n">
-        <v>0.051</v>
+        <v>0.008</v>
       </c>
       <c r="W45" t="n">
-        <v>968</v>
-      </c>
-      <c r="X45" t="inlineStr"/>
+        <v>5202</v>
+      </c>
+      <c r="X45" t="n">
+        <v>8.789999999999999</v>
+      </c>
       <c r="Y45" t="n">
-        <v>-2</v>
+        <v>43</v>
       </c>
       <c r="Z45" t="n">
-        <v>5</v>
+        <v>223</v>
       </c>
       <c r="AA45" t="n">
-        <v>-152</v>
+        <v>175</v>
       </c>
       <c r="AB45" t="n">
-        <v>-6.5</v>
+        <v>6.97</v>
       </c>
       <c r="AC45" t="n">
-        <v>9.24</v>
+        <v>21.4</v>
       </c>
       <c r="AD45" t="n">
-        <v>2.23</v>
+        <v>1.03</v>
       </c>
       <c r="AE45" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF45" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG45" t="n">
+        <v>360.16</v>
+      </c>
+      <c r="AH45" t="n">
+        <v>335.8</v>
+      </c>
+      <c r="AI45" t="n">
+        <v>13.8</v>
+      </c>
+      <c r="AJ45" t="n">
+        <v>335.4115036976171</v>
+      </c>
+      <c r="AK45" t="n">
+        <v>-5.4</v>
+      </c>
+      <c r="AL45" t="inlineStr">
+        <is>
+          <t>Aging</t>
+        </is>
+      </c>
+      <c r="AM45" t="inlineStr">
+        <is>
+          <t>Mature Accumulation</t>
+        </is>
+      </c>
+      <c r="AN45" t="inlineStr">
+        <is>
+          <t>Mature — Wait for Pullback</t>
+        </is>
+      </c>
+      <c r="AO45" t="inlineStr">
+        <is>
+          <t>30-06-2026</t>
+        </is>
+      </c>
+      <c r="AP45" t="inlineStr">
+        <is>
+          <t>18-08-2026</t>
+        </is>
+      </c>
+      <c r="AQ45" t="n">
+        <v>49</v>
+      </c>
+      <c r="AR45" t="n">
+        <v>94</v>
+      </c>
+      <c r="AS45" t="n">
+        <v>45</v>
+      </c>
+      <c r="AT45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW45" t="n">
         <v>1</v>
       </c>
-      <c r="AF45" t="n">
-        <v>6</v>
-      </c>
-      <c r="AG45" t="n">
-        <v>599.03</v>
-      </c>
-      <c r="AH45" t="n">
-        <v>549.9</v>
-      </c>
-      <c r="AI45" t="n">
-        <v>28.5</v>
-      </c>
-      <c r="AJ45" t="n">
-        <v>622.4351173945973</v>
-      </c>
-      <c r="AK45" t="n">
-        <v>-1.4</v>
-      </c>
-      <c r="AL45" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="AM45" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AN45" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO45" t="inlineStr">
-        <is>
-          <t>28-08-2026</t>
-        </is>
-      </c>
-      <c r="AP45" t="inlineStr">
-        <is>
-          <t>30-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ45" t="n">
-        <v>33</v>
-      </c>
-      <c r="AR45" t="n">
-        <v>35</v>
-      </c>
-      <c r="AS45" t="n">
-        <v>2</v>
-      </c>
-      <c r="AT45" t="n">
+      <c r="AX45" t="n">
         <v>1</v>
       </c>
-      <c r="AU45" t="n">
+      <c r="AY45" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB45" t="n">
+        <v>1094828</v>
+      </c>
+      <c r="BC45" t="n">
+        <v>1094828</v>
+      </c>
+      <c r="BD45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO45" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP45" t="n">
         <v>1</v>
       </c>
-      <c r="AV45" t="n">
-        <v>3</v>
-      </c>
-      <c r="AW45" t="n">
-        <v>4</v>
-      </c>
-      <c r="AX45" t="n">
-        <v>4</v>
-      </c>
-      <c r="AY45" t="n">
-        <v>2472736</v>
-      </c>
-      <c r="AZ45" t="n">
-        <v>2472736</v>
-      </c>
-      <c r="BA45" t="n">
-        <v>3760931</v>
-      </c>
-      <c r="BB45" t="n">
-        <v>4930931</v>
-      </c>
-      <c r="BC45" t="n">
-        <v>4930931</v>
-      </c>
-      <c r="BD45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM45" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN45" t="n">
-        <v>2472736</v>
-      </c>
-      <c r="BO45" t="n">
-        <v>3760931</v>
-      </c>
-      <c r="BP45" t="n">
-        <v>3</v>
-      </c>
       <c r="BQ45" t="n">
         <v>0</v>
       </c>
       <c r="BR45" t="n">
-        <v>0.6575</v>
+        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>MASFIN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>MAS Financial Services Limited</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -11042,40 +11042,40 @@
         </is>
       </c>
       <c r="E46" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F46" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="G46" t="n">
-        <v>9</v>
+        <v>0</v>
       </c>
       <c r="H46" t="n">
         <v>0</v>
       </c>
       <c r="I46" t="n">
-        <v>317.4</v>
+        <v>272.85</v>
       </c>
       <c r="J46" t="n">
-        <v>335.41</v>
+        <v>278.98</v>
       </c>
       <c r="K46" t="n">
-        <v>-5.4</v>
+        <v>-2.2</v>
       </c>
       <c r="L46" t="n">
-        <v>68.48</v>
+        <v>73.72</v>
       </c>
       <c r="M46" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="N46" t="n">
-        <v>4081958</v>
+        <v>2789837</v>
       </c>
       <c r="O46" t="n">
         <v>0</v>
       </c>
       <c r="P46" t="n">
-        <v>4081958</v>
+        <v>2789837</v>
       </c>
       <c r="Q46" t="n">
         <v>0</v>
@@ -11093,120 +11093,116 @@
       </c>
       <c r="U46" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
       <c r="V46" t="n">
-        <v>0.008</v>
+        <v>0.006</v>
       </c>
       <c r="W46" t="n">
-        <v>5199</v>
+        <v>4951</v>
       </c>
       <c r="X46" t="n">
-        <v>8.789999999999999</v>
+        <v>12.8</v>
       </c>
       <c r="Y46" t="n">
-        <v>43</v>
-      </c>
-      <c r="Z46" t="n">
-        <v>223</v>
-      </c>
+        <v>23</v>
+      </c>
+      <c r="Z46" t="inlineStr"/>
       <c r="AA46" t="n">
-        <v>175</v>
+        <v>21</v>
       </c>
       <c r="AB46" t="n">
-        <v>6.97</v>
+        <v>5.76</v>
       </c>
       <c r="AC46" t="n">
-        <v>21.4</v>
+        <v>11.3</v>
       </c>
       <c r="AD46" t="n">
-        <v>1.03</v>
+        <v>3.31</v>
       </c>
       <c r="AE46" t="b">
         <v>0</v>
       </c>
-      <c r="AF46" t="n">
+      <c r="AF46" t="inlineStr"/>
+      <c r="AG46" t="n">
+        <v>298.67</v>
+      </c>
+      <c r="AH46" t="n">
+        <v>311.73</v>
+      </c>
+      <c r="AI46" t="n">
+        <v>-2.4</v>
+      </c>
+      <c r="AJ46" t="n">
+        <v>278.9837</v>
+      </c>
+      <c r="AK46" t="n">
+        <v>-2.2</v>
+      </c>
+      <c r="AL46" t="inlineStr">
+        <is>
+          <t>Fresh</t>
+        </is>
+      </c>
+      <c r="AM46" t="inlineStr">
+        <is>
+          <t>Early Accumulation</t>
+        </is>
+      </c>
+      <c r="AN46" t="inlineStr">
+        <is>
+          <t>Early Accumulation</t>
+        </is>
+      </c>
+      <c r="AO46" t="inlineStr">
+        <is>
+          <t>25-09-2026</t>
+        </is>
+      </c>
+      <c r="AP46" t="inlineStr">
+        <is>
+          <t>29-09-2026</t>
+        </is>
+      </c>
+      <c r="AQ46" t="n">
+        <v>4</v>
+      </c>
+      <c r="AR46" t="n">
         <v>7</v>
       </c>
-      <c r="AG46" t="n">
-        <v>360.16</v>
-      </c>
-      <c r="AH46" t="n">
-        <v>335.8</v>
-      </c>
-      <c r="AI46" t="n">
-        <v>13.8</v>
-      </c>
-      <c r="AJ46" t="n">
-        <v>335.4115036976171</v>
-      </c>
-      <c r="AK46" t="n">
-        <v>-5.4</v>
-      </c>
-      <c r="AL46" t="inlineStr">
-        <is>
-          <t>Aging</t>
-        </is>
-      </c>
-      <c r="AM46" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN46" t="inlineStr">
-        <is>
-          <t>Mature — Wait for Pullback</t>
-        </is>
-      </c>
-      <c r="AO46" t="inlineStr">
-        <is>
-          <t>30-06-2026</t>
-        </is>
-      </c>
-      <c r="AP46" t="inlineStr">
-        <is>
-          <t>18-08-2026</t>
-        </is>
-      </c>
-      <c r="AQ46" t="n">
-        <v>49</v>
-      </c>
-      <c r="AR46" t="n">
-        <v>94</v>
-      </c>
       <c r="AS46" t="n">
-        <v>45</v>
+        <v>3</v>
       </c>
       <c r="AT46" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AU46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AV46" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AW46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AX46" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AY46" t="n">
-        <v>0</v>
+        <v>1390000</v>
       </c>
       <c r="AZ46" t="n">
-        <v>0</v>
+        <v>2789837</v>
       </c>
       <c r="BA46" t="n">
-        <v>0</v>
+        <v>2789837</v>
       </c>
       <c r="BB46" t="n">
-        <v>1094828</v>
+        <v>2789837</v>
       </c>
       <c r="BC46" t="n">
-        <v>1094828</v>
+        <v>2789837</v>
       </c>
       <c r="BD46" t="n">
         <v>0</v>
@@ -11239,10 +11235,10 @@
         <v>0</v>
       </c>
       <c r="BN46" t="n">
-        <v>0</v>
+        <v>1390000</v>
       </c>
       <c r="BO46" t="n">
-        <v>0</v>
+        <v>2789837</v>
       </c>
       <c r="BP46" t="n">
         <v>1</v>
@@ -11251,235 +11247,239 @@
         <v>0</v>
       </c>
       <c r="BR46" t="n">
-        <v>0</v>
+        <v>0.4982</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MASFIN</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MAS Financial Services Limited</t>
+          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>0</v>
+      </c>
+      <c r="F47" t="n">
+        <v>14</v>
+      </c>
+      <c r="G47" t="n">
+        <v>25</v>
+      </c>
+      <c r="H47" t="n">
+        <v>-19</v>
+      </c>
+      <c r="I47" t="n">
+        <v>1766.5</v>
+      </c>
+      <c r="J47" t="n">
+        <v>1579.83</v>
+      </c>
+      <c r="K47" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="L47" t="n">
+        <v>67.55</v>
+      </c>
+      <c r="M47" t="n">
+        <v>12.76</v>
+      </c>
+      <c r="N47" t="n">
+        <v>127601332</v>
+      </c>
+      <c r="O47" t="n">
+        <v>130031492</v>
+      </c>
+      <c r="P47" t="n">
+        <v>-2430160</v>
+      </c>
+      <c r="Q47" t="n">
+        <v>101.9</v>
+      </c>
+      <c r="R47" t="inlineStr">
+        <is>
+          <t>Net Selling</t>
+        </is>
+      </c>
+      <c r="S47" t="b">
+        <v>0</v>
+      </c>
+      <c r="T47" t="n">
+        <v>3</v>
+      </c>
+      <c r="U47" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="V47" t="n">
+        <v>0</v>
+      </c>
+      <c r="W47" t="n">
+        <v>3686</v>
+      </c>
+      <c r="X47" t="n">
+        <v>83</v>
+      </c>
+      <c r="Y47" t="n">
+        <v>42</v>
+      </c>
+      <c r="Z47" t="n">
         <v>13</v>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E47" t="n">
-        <v>6</v>
-      </c>
-      <c r="F47" t="n">
-        <v>7</v>
-      </c>
-      <c r="G47" t="n">
-        <v>0</v>
-      </c>
-      <c r="H47" t="n">
-        <v>0</v>
-      </c>
-      <c r="I47" t="n">
-        <v>272.85</v>
-      </c>
-      <c r="J47" t="n">
-        <v>278.98</v>
-      </c>
-      <c r="K47" t="n">
-        <v>-2.2</v>
-      </c>
-      <c r="L47" t="n">
-        <v>73.72</v>
-      </c>
-      <c r="M47" t="n">
-        <v>0.28</v>
-      </c>
-      <c r="N47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="O47" t="n">
-        <v>0</v>
-      </c>
-      <c r="P47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="Q47" t="n">
-        <v>0</v>
-      </c>
-      <c r="R47" t="inlineStr">
-        <is>
-          <t>Net Buying</t>
-        </is>
-      </c>
-      <c r="S47" t="b">
-        <v>0</v>
-      </c>
-      <c r="T47" t="n">
+      <c r="AA47" t="n">
+        <v>22</v>
+      </c>
+      <c r="AB47" t="n">
+        <v>5.05</v>
+      </c>
+      <c r="AC47" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="AD47" t="n">
+        <v>0.03</v>
+      </c>
+      <c r="AE47" t="b">
+        <v>0</v>
+      </c>
+      <c r="AF47" t="n">
+        <v>27</v>
+      </c>
+      <c r="AG47" t="n">
+        <v>1648.79</v>
+      </c>
+      <c r="AH47" t="n">
+        <v>1391.54</v>
+      </c>
+      <c r="AI47" t="n">
+        <v>84.09999999999999</v>
+      </c>
+      <c r="AJ47" t="n">
+        <v>1579.830529039607</v>
+      </c>
+      <c r="AK47" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="AL47" t="inlineStr">
+        <is>
+          <t>Stale</t>
+        </is>
+      </c>
+      <c r="AM47" t="inlineStr">
+        <is>
+          <t>Stale Accumulation</t>
+        </is>
+      </c>
+      <c r="AN47" t="inlineStr">
+        <is>
+          <t>Late — Poor Entry</t>
+        </is>
+      </c>
+      <c r="AO47" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AP47" t="inlineStr">
+        <is>
+          <t>25-06-2026</t>
+        </is>
+      </c>
+      <c r="AQ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AR47" t="n">
+        <v>99</v>
+      </c>
+      <c r="AS47" t="n">
+        <v>99</v>
+      </c>
+      <c r="AT47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AU47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AV47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AW47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AX47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AY47" t="n">
+        <v>0</v>
+      </c>
+      <c r="AZ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BC47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BD47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BG47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BH47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BI47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BM47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO47" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP47" t="n">
         <v>2</v>
       </c>
-      <c r="U47" t="inlineStr">
-        <is>
-          <t>29-09-2026</t>
-        </is>
-      </c>
-      <c r="V47" t="n">
-        <v>0.006</v>
-      </c>
-      <c r="W47" t="n">
-        <v>4942</v>
-      </c>
-      <c r="X47" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="Y47" t="n">
-        <v>23</v>
-      </c>
-      <c r="Z47" t="inlineStr"/>
-      <c r="AA47" t="n">
-        <v>21</v>
-      </c>
-      <c r="AB47" t="n">
-        <v>5.76</v>
-      </c>
-      <c r="AC47" t="n">
-        <v>11.3</v>
-      </c>
-      <c r="AD47" t="n">
-        <v>3.31</v>
-      </c>
-      <c r="AE47" t="b">
-        <v>0</v>
-      </c>
-      <c r="AF47" t="inlineStr"/>
-      <c r="AG47" t="n">
-        <v>298.67</v>
-      </c>
-      <c r="AH47" t="n">
-        <v>311.73</v>
-      </c>
-      <c r="AI47" t="n">
-        <v>-2.4</v>
-      </c>
-      <c r="AJ47" t="n">
-        <v>278.9837</v>
-      </c>
-      <c r="AK47" t="n">
-        <v>-2.2</v>
-      </c>
-      <c r="AL47" t="inlineStr">
-        <is>
-          <t>Fresh</t>
-        </is>
-      </c>
-      <c r="AM47" t="inlineStr">
-        <is>
-          <t>Early Accumulation</t>
-        </is>
-      </c>
-      <c r="AN47" t="inlineStr">
-        <is>
-          <t>Early Accumulation</t>
-        </is>
-      </c>
-      <c r="AO47" t="inlineStr">
-        <is>
-          <t>25-09-2026</t>
-        </is>
-      </c>
-      <c r="AP47" t="inlineStr">
-        <is>
-          <t>29-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ47" t="n">
-        <v>4</v>
-      </c>
-      <c r="AR47" t="n">
-        <v>7</v>
-      </c>
-      <c r="AS47" t="n">
-        <v>3</v>
-      </c>
-      <c r="AT47" t="n">
+      <c r="BQ47" t="n">
         <v>1</v>
       </c>
-      <c r="AU47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AV47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AW47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AX47" t="n">
-        <v>2</v>
-      </c>
-      <c r="AY47" t="n">
-        <v>1390000</v>
-      </c>
-      <c r="AZ47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="BA47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="BB47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="BC47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="BD47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BH47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM47" t="n">
-        <v>0</v>
-      </c>
-      <c r="BN47" t="n">
-        <v>1390000</v>
-      </c>
-      <c r="BO47" t="n">
-        <v>2789837</v>
-      </c>
-      <c r="BP47" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ47" t="n">
-        <v>0</v>
-      </c>
       <c r="BR47" t="n">
-        <v>0.4982</v>
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -11560,7 +11560,7 @@
         <v>0</v>
       </c>
       <c r="W48" t="n">
-        <v>8633</v>
+        <v>8637</v>
       </c>
       <c r="X48" t="n">
         <v>14.6</v>
@@ -11717,158 +11717,158 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C49" t="n">
+        <v>3</v>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Avoid</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>4</v>
+      </c>
+      <c r="F49" t="n">
         <v>5</v>
       </c>
-      <c r="D49" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E49" t="n">
-        <v>0</v>
-      </c>
-      <c r="F49" t="n">
-        <v>14</v>
-      </c>
       <c r="G49" t="n">
-        <v>25</v>
+        <v>5</v>
       </c>
       <c r="H49" t="n">
-        <v>-19</v>
+        <v>-1</v>
       </c>
       <c r="I49" t="n">
-        <v>1766.5</v>
+        <v>108.85</v>
       </c>
       <c r="J49" t="n">
-        <v>789.9400000000001</v>
+        <v>111.01</v>
       </c>
       <c r="K49" t="n">
-        <v>123.6</v>
+        <v>-1.9</v>
       </c>
       <c r="L49" t="n">
-        <v>67.55</v>
+        <v>73.48</v>
       </c>
       <c r="M49" t="n">
-        <v>12.76</v>
+        <v>0.45</v>
       </c>
       <c r="N49" t="n">
-        <v>127606073</v>
+        <v>4484713</v>
       </c>
       <c r="O49" t="n">
-        <v>130033072</v>
+        <v>0</v>
       </c>
       <c r="P49" t="n">
-        <v>-2426999</v>
+        <v>4484713</v>
       </c>
       <c r="Q49" t="n">
-        <v>101.9</v>
+        <v>0</v>
       </c>
       <c r="R49" t="inlineStr">
         <is>
-          <t>Net Selling</t>
+          <t>Net Buying</t>
         </is>
       </c>
       <c r="S49" t="b">
         <v>0</v>
       </c>
       <c r="T49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="U49" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="V49" t="n">
-        <v>0</v>
+        <v>0.218</v>
       </c>
       <c r="W49" t="n">
-        <v>3727</v>
+        <v>206</v>
       </c>
       <c r="X49" t="n">
-        <v>83.90000000000001</v>
+        <v>24.6</v>
       </c>
       <c r="Y49" t="n">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="Z49" t="n">
-        <v>13</v>
+        <v>12.07</v>
       </c>
       <c r="AA49" t="n">
-        <v>22</v>
+        <v>-29</v>
       </c>
       <c r="AB49" t="n">
-        <v>5.05</v>
+        <v>1.02</v>
       </c>
       <c r="AC49" t="n">
-        <v>19.9</v>
+        <v>7.92</v>
       </c>
       <c r="AD49" t="n">
-        <v>0.03</v>
+        <v>0.98</v>
       </c>
       <c r="AE49" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AF49" t="n">
-        <v>27</v>
+        <v>4.11</v>
       </c>
       <c r="AG49" t="n">
-        <v>1648.79</v>
+        <v>112.05</v>
       </c>
       <c r="AH49" t="n">
-        <v>1391.54</v>
+        <v>117.93</v>
       </c>
       <c r="AI49" t="n">
-        <v>84.09999999999999</v>
+        <v>6.5</v>
       </c>
       <c r="AJ49" t="n">
-        <v>789.9446136512771</v>
+        <v>111.0077475247525</v>
       </c>
       <c r="AK49" t="n">
-        <v>123.6</v>
+        <v>-1.9</v>
       </c>
       <c r="AL49" t="inlineStr">
         <is>
-          <t>Stale</t>
+          <t>Active</t>
         </is>
       </c>
       <c r="AM49" t="inlineStr">
         <is>
-          <t>Stale Accumulation</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AN49" t="inlineStr">
         <is>
-          <t>Late — Poor Entry</t>
+          <t>Confirmed Accumulation</t>
         </is>
       </c>
       <c r="AO49" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>17-08-2026</t>
         </is>
       </c>
       <c r="AP49" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AQ49" t="n">
-        <v>0</v>
+        <v>17</v>
       </c>
       <c r="AR49" t="n">
-        <v>99</v>
+        <v>46</v>
       </c>
       <c r="AS49" t="n">
-        <v>99</v>
+        <v>29</v>
       </c>
       <c r="AT49" t="n">
         <v>0</v>
@@ -11877,13 +11877,13 @@
         <v>0</v>
       </c>
       <c r="AV49" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AW49" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AX49" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AY49" t="n">
         <v>0</v>
@@ -11892,13 +11892,13 @@
         <v>0</v>
       </c>
       <c r="BA49" t="n">
-        <v>0</v>
+        <v>207193</v>
       </c>
       <c r="BB49" t="n">
-        <v>0</v>
+        <v>4484713</v>
       </c>
       <c r="BC49" t="n">
-        <v>0</v>
+        <v>4484713</v>
       </c>
       <c r="BD49" t="n">
         <v>0</v>
@@ -11934,13 +11934,13 @@
         <v>0</v>
       </c>
       <c r="BO49" t="n">
-        <v>0</v>
+        <v>207193</v>
       </c>
       <c r="BP49" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="BQ49" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="BR49" t="n">
         <v>0</v>
@@ -11949,16 +11949,16 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>JINDAL STEEL LIMITED</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="D50" t="inlineStr">
         <is>
@@ -11966,54 +11966,54 @@
         </is>
       </c>
       <c r="E50" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="F50" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="G50" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="H50" t="n">
-        <v>-1</v>
+        <v>-18</v>
       </c>
       <c r="I50" t="n">
-        <v>108.85</v>
+        <v>1100.5</v>
       </c>
       <c r="J50" t="n">
-        <v>111.01</v>
+        <v>1157.18</v>
       </c>
       <c r="K50" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="L50" t="n">
-        <v>73.48</v>
+        <v>61.21</v>
       </c>
       <c r="M50" t="n">
-        <v>0.45</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="N50" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="O50" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="P50" t="n">
-        <v>4484713</v>
+        <v>-16092588</v>
       </c>
       <c r="Q50" t="n">
-        <v>0</v>
+        <v>117.47</v>
       </c>
       <c r="R50" t="inlineStr">
         <is>
-          <t>Net Buying</t>
+          <t>Net Selling</t>
         </is>
       </c>
       <c r="S50" t="b">
         <v>0</v>
       </c>
       <c r="T50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="U50" t="inlineStr">
         <is>
@@ -12021,52 +12021,52 @@
         </is>
       </c>
       <c r="V50" t="n">
-        <v>0.222</v>
+        <v>0</v>
       </c>
       <c r="W50" t="n">
-        <v>202</v>
+        <v>112261</v>
       </c>
       <c r="X50" t="n">
-        <v>24.1</v>
+        <v>32.3</v>
       </c>
       <c r="Y50" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="Z50" t="n">
-        <v>12.07</v>
+        <v>2224</v>
       </c>
       <c r="AA50" t="n">
-        <v>-29</v>
+        <v>-28</v>
       </c>
       <c r="AB50" t="n">
-        <v>1.02</v>
+        <v>10.65</v>
       </c>
       <c r="AC50" t="n">
-        <v>7.92</v>
+        <v>10.8</v>
       </c>
       <c r="AD50" t="n">
-        <v>0.98</v>
+        <v>0.16</v>
       </c>
       <c r="AE50" t="b">
         <v>1</v>
       </c>
       <c r="AF50" t="n">
-        <v>4.11</v>
+        <v>15</v>
       </c>
       <c r="AG50" t="n">
-        <v>112.05</v>
+        <v>1123.81</v>
       </c>
       <c r="AH50" t="n">
-        <v>117.93</v>
+        <v>1135.91</v>
       </c>
       <c r="AI50" t="n">
-        <v>6.5</v>
+        <v>-1.1</v>
       </c>
       <c r="AJ50" t="n">
-        <v>111.0077475247525</v>
+        <v>1157.177537688442</v>
       </c>
       <c r="AK50" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="AL50" t="inlineStr">
         <is>
@@ -12075,17 +12075,17 @@
       </c>
       <c r="AM50" t="inlineStr">
         <is>
+          <t>Mature Accumulation</t>
+        </is>
+      </c>
+      <c r="AN50" t="inlineStr">
+        <is>
           <t>Confirmed Accumulation</t>
         </is>
       </c>
-      <c r="AN50" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
       <c r="AO50" t="inlineStr">
         <is>
-          <t>17-08-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
       <c r="AP50" t="inlineStr">
@@ -12094,10 +12094,10 @@
         </is>
       </c>
       <c r="AQ50" t="n">
-        <v>17</v>
+        <v>0</v>
       </c>
       <c r="AR50" t="n">
-        <v>46</v>
+        <v>29</v>
       </c>
       <c r="AS50" t="n">
         <v>29</v>
@@ -12112,10 +12112,10 @@
         <v>1</v>
       </c>
       <c r="AW50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AX50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="AY50" t="n">
         <v>0</v>
@@ -12124,13 +12124,13 @@
         <v>0</v>
       </c>
       <c r="BA50" t="n">
-        <v>207193</v>
+        <v>92111332</v>
       </c>
       <c r="BB50" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="BC50" t="n">
-        <v>4484713</v>
+        <v>92111332</v>
       </c>
       <c r="BD50" t="n">
         <v>0</v>
@@ -12142,10 +12142,10 @@
         <v>0</v>
       </c>
       <c r="BG50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BH50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI50" t="n">
         <v>0</v>
@@ -12157,256 +12157,24 @@
         <v>0</v>
       </c>
       <c r="BL50" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="BM50" t="n">
-        <v>0</v>
+        <v>108203920</v>
       </c>
       <c r="BN50" t="n">
         <v>0</v>
       </c>
       <c r="BO50" t="n">
-        <v>207193</v>
+        <v>92111332</v>
       </c>
       <c r="BP50" t="n">
         <v>1</v>
       </c>
       <c r="BQ50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BR50" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>JINDAL STEEL LIMITED</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>0</v>
-      </c>
-      <c r="D51" t="inlineStr">
-        <is>
-          <t>Avoid</t>
-        </is>
-      </c>
-      <c r="E51" t="n">
-        <v>0</v>
-      </c>
-      <c r="F51" t="n">
-        <v>12</v>
-      </c>
-      <c r="G51" t="n">
-        <v>0</v>
-      </c>
-      <c r="H51" t="n">
-        <v>-18</v>
-      </c>
-      <c r="I51" t="n">
-        <v>1100.5</v>
-      </c>
-      <c r="J51" t="n">
-        <v>1157.18</v>
-      </c>
-      <c r="K51" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="L51" t="n">
-        <v>61.21</v>
-      </c>
-      <c r="M51" t="n">
-        <v>9.210000000000001</v>
-      </c>
-      <c r="N51" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="O51" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="P51" t="n">
-        <v>-16092588</v>
-      </c>
-      <c r="Q51" t="n">
-        <v>117.47</v>
-      </c>
-      <c r="R51" t="inlineStr">
-        <is>
-          <t>Net Selling</t>
-        </is>
-      </c>
-      <c r="S51" t="b">
-        <v>0</v>
-      </c>
-      <c r="T51" t="n">
-        <v>1</v>
-      </c>
-      <c r="U51" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="V51" t="n">
-        <v>0</v>
-      </c>
-      <c r="W51" t="n">
-        <v>112548</v>
-      </c>
-      <c r="X51" t="n">
-        <v>32.4</v>
-      </c>
-      <c r="Y51" t="n">
-        <v>18</v>
-      </c>
-      <c r="Z51" t="n">
-        <v>2224</v>
-      </c>
-      <c r="AA51" t="n">
-        <v>-28</v>
-      </c>
-      <c r="AB51" t="n">
-        <v>10.65</v>
-      </c>
-      <c r="AC51" t="n">
-        <v>10.8</v>
-      </c>
-      <c r="AD51" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AE51" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF51" t="n">
-        <v>15</v>
-      </c>
-      <c r="AG51" t="n">
-        <v>1123.81</v>
-      </c>
-      <c r="AH51" t="n">
-        <v>1135.91</v>
-      </c>
-      <c r="AI51" t="n">
-        <v>-1.1</v>
-      </c>
-      <c r="AJ51" t="n">
-        <v>1157.177537688442</v>
-      </c>
-      <c r="AK51" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="AL51" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
-      <c r="AM51" t="inlineStr">
-        <is>
-          <t>Mature Accumulation</t>
-        </is>
-      </c>
-      <c r="AN51" t="inlineStr">
-        <is>
-          <t>Confirmed Accumulation</t>
-        </is>
-      </c>
-      <c r="AO51" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="AP51" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-      <c r="AQ51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR51" t="n">
-        <v>29</v>
-      </c>
-      <c r="AS51" t="n">
-        <v>29</v>
-      </c>
-      <c r="AT51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AU51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AW51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AX51" t="n">
-        <v>1</v>
-      </c>
-      <c r="AY51" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BA51" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BB51" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BC51" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BD51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BH51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BI51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BJ51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BL51" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="BM51" t="n">
-        <v>108203920</v>
-      </c>
-      <c r="BN51" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO51" t="n">
-        <v>92111332</v>
-      </c>
-      <c r="BP51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BQ51" t="n">
-        <v>1</v>
-      </c>
-      <c r="BR51" t="n">
         <v>0</v>
       </c>
     </row>
@@ -12421,7 +12189,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13745,350 +13513,350 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>MAHSEAMLES</t>
+          <t>INDIQUBE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Maharashtra Seamless Limited</t>
+          <t>Indiqube Spaces Limited</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>698.75</v>
+        <v>197.49</v>
       </c>
       <c r="D38" t="n">
-        <v>618.78</v>
+        <v>195.05</v>
       </c>
       <c r="E38" t="n">
-        <v>12.9</v>
+        <v>1.3</v>
       </c>
       <c r="F38" t="n">
-        <v>67.86</v>
+        <v>60.6</v>
       </c>
       <c r="G38" t="n">
-        <v>102.7</v>
+        <v>0.45</v>
       </c>
       <c r="H38" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>30-06-2026</t>
+          <t>25-09-2026</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>INDIQUBE</t>
+          <t>UYFINCORP</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Indiqube Spaces Limited</t>
+          <t>U. Y. Fincorp Limited</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>197.49</v>
+        <v>22.86</v>
       </c>
       <c r="D39" t="n">
-        <v>195.05</v>
+        <v>21.01</v>
       </c>
       <c r="E39" t="n">
-        <v>1.3</v>
+        <v>8.800000000000001</v>
       </c>
       <c r="F39" t="n">
-        <v>60.6</v>
+        <v>70.87</v>
       </c>
       <c r="G39" t="n">
-        <v>0.45</v>
+        <v>0.5</v>
       </c>
       <c r="H39" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>25-09-2026</t>
+          <t>19-08-2026</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>UYFINCORP</t>
+          <t>SOTL</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>U. Y. Fincorp Limited</t>
+          <t>Savita Oil Technologies Limited</t>
         </is>
       </c>
       <c r="C40" t="n">
-        <v>22.86</v>
+        <v>729.5</v>
       </c>
       <c r="D40" t="n">
-        <v>21.01</v>
+        <v>726.25</v>
       </c>
       <c r="E40" t="n">
-        <v>8.800000000000001</v>
+        <v>0.4</v>
       </c>
       <c r="F40" t="n">
-        <v>70.87</v>
+        <v>71.92</v>
       </c>
       <c r="G40" t="n">
-        <v>0.5</v>
+        <v>3.76</v>
       </c>
       <c r="H40" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>19-08-2026</t>
+          <t>24-09-2026</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SOTL</t>
+          <t>ASAHISONG</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Savita Oil Technologies Limited</t>
+          <t>ASAHI SONGWON COLORS LIMITED</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>729.5</v>
+        <v>371.25</v>
       </c>
       <c r="D41" t="n">
-        <v>726.25</v>
+        <v>338.1</v>
       </c>
       <c r="E41" t="n">
-        <v>0.4</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="F41" t="n">
-        <v>71.92</v>
+        <v>66.73</v>
       </c>
       <c r="G41" t="n">
-        <v>3.76</v>
+        <v>0.34</v>
       </c>
       <c r="H41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I41" t="inlineStr">
         <is>
-          <t>24-09-2026</t>
+          <t>11-08-2026</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ASAHISONG</t>
+          <t>HINDCON</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ASAHI SONGWON COLORS LIMITED</t>
+          <t>Hindcon Chemicals Limited</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>371.25</v>
+        <v>33.3</v>
       </c>
       <c r="D42" t="n">
-        <v>338.1</v>
+        <v>23.55</v>
       </c>
       <c r="E42" t="n">
-        <v>9.800000000000001</v>
+        <v>41.4</v>
       </c>
       <c r="F42" t="n">
-        <v>66.73</v>
+        <v>68.34</v>
       </c>
       <c r="G42" t="n">
-        <v>0.34</v>
+        <v>0.2</v>
       </c>
       <c r="H42" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>11-08-2026</t>
+          <t>23-09-2026</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HINDCON</t>
+          <t>CHEMBOND</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Hindcon Chemicals Limited</t>
+          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>33.3</v>
+        <v>177.64</v>
       </c>
       <c r="D43" t="n">
-        <v>23.55</v>
+        <v>170.45</v>
       </c>
       <c r="E43" t="n">
-        <v>41.4</v>
+        <v>4.2</v>
       </c>
       <c r="F43" t="n">
-        <v>68.34</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G43" t="n">
-        <v>0.2</v>
+        <v>0.26</v>
       </c>
       <c r="H43" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>23-09-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CHEMBOND</t>
+          <t>SGIL</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CHEMBOND MATERIAL TECHNOLOGIES LIMITED</t>
+          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>177.64</v>
+        <v>613.85</v>
       </c>
       <c r="D44" t="n">
-        <v>170.45</v>
+        <v>622.4400000000001</v>
       </c>
       <c r="E44" t="n">
-        <v>4.2</v>
+        <v>-1.4</v>
       </c>
       <c r="F44" t="n">
-        <v>67.54000000000001</v>
+        <v>74.02</v>
       </c>
       <c r="G44" t="n">
-        <v>0.26</v>
+        <v>0.49</v>
       </c>
       <c r="H44" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>03-09-2026</t>
+          <t>30-09-2026</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>SGIL</t>
+          <t>SENCO</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SYNERGY GREEN INDUSTRIES LIMITED</t>
+          <t>SENCO GOLD LIMITED</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>613.85</v>
+        <v>317.4</v>
       </c>
       <c r="D45" t="n">
-        <v>622.4400000000001</v>
+        <v>335.41</v>
       </c>
       <c r="E45" t="n">
-        <v>-1.4</v>
+        <v>-5.4</v>
       </c>
       <c r="F45" t="n">
-        <v>74.02</v>
+        <v>68.48</v>
       </c>
       <c r="G45" t="n">
-        <v>0.49</v>
+        <v>0.41</v>
       </c>
       <c r="H45" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>30-09-2026</t>
+          <t>18-08-2026</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>SENCO</t>
+          <t>MASFIN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>SENCO GOLD LIMITED</t>
+          <t>MAS Financial Services Limited</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>317.4</v>
+        <v>272.85</v>
       </c>
       <c r="D46" t="n">
-        <v>335.41</v>
+        <v>278.98</v>
       </c>
       <c r="E46" t="n">
-        <v>-5.4</v>
+        <v>-2.2</v>
       </c>
       <c r="F46" t="n">
-        <v>68.48</v>
+        <v>73.72</v>
       </c>
       <c r="G46" t="n">
-        <v>0.41</v>
+        <v>0.28</v>
       </c>
       <c r="H46" t="n">
         <v>2</v>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>18-08-2026</t>
+          <t>29-09-2026</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>MASFIN</t>
+          <t>NPST</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MAS Financial Services Limited</t>
+          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>272.85</v>
+        <v>1766.5</v>
       </c>
       <c r="D47" t="n">
-        <v>278.98</v>
+        <v>1579.83</v>
       </c>
       <c r="E47" t="n">
-        <v>-2.2</v>
+        <v>11.8</v>
       </c>
       <c r="F47" t="n">
-        <v>73.72</v>
+        <v>67.55</v>
       </c>
       <c r="G47" t="n">
-        <v>0.28</v>
+        <v>12.76</v>
       </c>
       <c r="H47" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>29-09-2026</t>
+          <t>25-06-2026</t>
         </is>
       </c>
     </row>
@@ -14130,103 +13898,68 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>NPST</t>
+          <t>VSTL</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>NETWORK PEOPLE SERVICES TECHNOLOGIES LIMITED</t>
+          <t>VIBHOR STEEL TUBES LIMITED</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>1766.5</v>
+        <v>108.85</v>
       </c>
       <c r="D49" t="n">
-        <v>789.9400000000001</v>
+        <v>111.01</v>
       </c>
       <c r="E49" t="n">
-        <v>123.6</v>
+        <v>-1.9</v>
       </c>
       <c r="F49" t="n">
-        <v>67.55</v>
+        <v>73.48</v>
       </c>
       <c r="G49" t="n">
-        <v>12.76</v>
+        <v>0.45</v>
       </c>
       <c r="H49" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>25-06-2026</t>
+          <t>03-09-2026</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>VSTL</t>
+          <t>JINDALSTEL</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>VIBHOR STEEL TUBES LIMITED</t>
+          <t>JINDAL STEEL LIMITED</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>108.85</v>
+        <v>1100.5</v>
       </c>
       <c r="D50" t="n">
-        <v>111.01</v>
+        <v>1157.18</v>
       </c>
       <c r="E50" t="n">
-        <v>-1.9</v>
+        <v>-4.9</v>
       </c>
       <c r="F50" t="n">
-        <v>73.48</v>
+        <v>61.21</v>
       </c>
       <c r="G50" t="n">
-        <v>0.45</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="H50" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="I50" t="inlineStr">
-        <is>
-          <t>03-09-2026</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" t="inlineStr">
-        <is>
-          <t>JINDALSTEL</t>
-        </is>
-      </c>
-      <c r="B51" t="inlineStr">
-        <is>
-          <t>JINDAL STEEL LIMITED</t>
-        </is>
-      </c>
-      <c r="C51" t="n">
-        <v>1100.5</v>
-      </c>
-      <c r="D51" t="n">
-        <v>1157.18</v>
-      </c>
-      <c r="E51" t="n">
-        <v>-4.9</v>
-      </c>
-      <c r="F51" t="n">
-        <v>61.21</v>
-      </c>
-      <c r="G51" t="n">
-        <v>9.210000000000001</v>
-      </c>
-      <c r="H51" t="n">
-        <v>1</v>
-      </c>
-      <c r="I51" t="inlineStr">
         <is>
           <t>03-09-2026</t>
         </is>
@@ -14295,7 +14028,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -14315,7 +14048,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">

</xml_diff>